<commit_message>
Refactor case management forms to remove secondary intake fields
- Removed all references to secondary identifying and victim fields from the case mapping functions in useCases.js and useCasesOffline.js.
- Updated case payload construction in caseSubmission.js to eliminate handling of secondary intake data.
- Simplified family member handling in case management forms by merging family members into a single group.
- Adjusted the IntakeSheetCaseCreate and IntakeSheetCaseEdit components to reflect the removal of secondary data fields and updated the tab navigation accordingly.
- Cleaned up the Excel export functionality to exclude secondary fields.
</commit_message>
<xml_diff>
--- a/public/excel-templates/case-template.xlsx
+++ b/public/excel-templates/case-template.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -475,13 +475,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="24">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <color theme="1"/>
+      <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <i/>
@@ -496,28 +497,21 @@
     </font>
     <font>
       <b/>
-      <sz val="24.0"/>
       <color theme="1"/>
+      <sz val="24"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <u/>
-      <sz val="9.0"/>
       <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="9.0"/>
-      <color theme="1"/>
+      <sz val="9"/>
       <name val="Arial"/>
     </font>
     <font>
       <u/>
-      <sz val="9.0"/>
       <color theme="1"/>
+      <sz val="9"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -532,19 +526,13 @@
     </font>
     <font>
       <u/>
-      <sz val="9.0"/>
       <color theme="1"/>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
-      <u/>
-      <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10.0"/>
-      <color theme="1"/>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -553,71 +541,21 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11.0"/>
       <color rgb="FF000000"/>
+      <sz val="11"/>
       <name val="'Google Sans Text'"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="9.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="9.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="9.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
     </font>
     <font>
       <b/>
       <i/>
       <u/>
-      <sz val="9.0"/>
       <color theme="1"/>
+      <sz val="9"/>
       <name val="Arial"/>
     </font>
     <font>
-      <b/>
-      <i/>
-      <u/>
-      <sz val="9.0"/>
       <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <u/>
-      <sz val="9.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="9.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <u/>
-      <sz val="9.0"/>
-      <color theme="1"/>
+      <sz val="9"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -626,7 +564,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -648,58 +586,88 @@
     </fill>
   </fills>
   <borders count="13">
-    <border/>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-    </border>
-    <border>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -709,19 +677,27 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -736,158 +712,161 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="52">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="11" fillId="3" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="11" fillId="4" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="11" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="11" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="6" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="11" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="6" fillId="2" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="7" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="8" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="0" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="12" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="2" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="10" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1085,49 +1064,80 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:H117"/>
+  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="12.63" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="22.0"/>
-    <col customWidth="1" min="2" max="2" width="22.88"/>
-    <col customWidth="1" min="3" max="3" width="22.63"/>
-    <col customWidth="1" min="4" max="4" width="23.5"/>
-    <col customWidth="1" min="5" max="5" width="27.0"/>
-    <col customWidth="1" min="6" max="6" width="30.13"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="22.88" customWidth="1"/>
+    <col min="3" max="3" width="22.63" customWidth="1"/>
+    <col min="4" max="4" width="23.5" customWidth="1"/>
+    <col min="5" max="5" width="27" customWidth="1"/>
+    <col min="6" max="6" width="30.13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1"/>
+      <c r="C1"/>
+      <c r="D1"/>
+      <c r="E1"/>
+      <c r="F1"/>
+      <c r="G1"/>
       <c r="H1" s="2"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2"/>
+      <c r="C2"/>
+      <c r="D2"/>
+      <c r="E2"/>
+      <c r="F2"/>
+      <c r="G2"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3"/>
+      <c r="C3"/>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3"/>
+      <c r="G3"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
+      <c r="B4"/>
+      <c r="C4"/>
+      <c r="D4"/>
+      <c r="E4"/>
+      <c r="F4"/>
+      <c r="G4"/>
       <c r="H4" s="2"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
+      <c r="B5"/>
+      <c r="C5"/>
+      <c r="D5"/>
+      <c r="E5"/>
+      <c r="F5"/>
+      <c r="G5"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
@@ -1139,15 +1149,27 @@
       <c r="G6" s="5"/>
       <c r="H6" s="6"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="7"/>
+      <c r="B7"/>
+      <c r="C7"/>
+      <c r="D7"/>
+      <c r="E7"/>
+      <c r="F7"/>
+      <c r="G7"/>
       <c r="H7" s="2"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
+      <c r="B8"/>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
       <c r="H8" s="2"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>5</v>
       </c>
@@ -1159,7 +1181,7 @@
       <c r="G9" s="9"/>
       <c r="H9" s="10"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>6</v>
       </c>
@@ -1173,7 +1195,7 @@
       <c r="G10" s="9"/>
       <c r="H10" s="10"/>
     </row>
-    <row r="11">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -1187,7 +1209,7 @@
       <c r="G11" s="9"/>
       <c r="H11" s="10"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>10</v>
       </c>
@@ -1201,7 +1223,7 @@
       <c r="G12" s="9"/>
       <c r="H12" s="10"/>
     </row>
-    <row r="13">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>12</v>
       </c>
@@ -1215,7 +1237,7 @@
       <c r="G13" s="9"/>
       <c r="H13" s="10"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="s">
         <v>14</v>
       </c>
@@ -1229,7 +1251,7 @@
       <c r="G14" s="9"/>
       <c r="H14" s="10"/>
     </row>
-    <row r="15">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
         <v>16</v>
       </c>
@@ -1243,7 +1265,7 @@
       <c r="G15" s="9"/>
       <c r="H15" s="10"/>
     </row>
-    <row r="16">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
         <v>18</v>
       </c>
@@ -1257,7 +1279,7 @@
       <c r="G16" s="9"/>
       <c r="H16" s="10"/>
     </row>
-    <row r="17">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>20</v>
       </c>
@@ -1271,7 +1293,7 @@
       <c r="G17" s="9"/>
       <c r="H17" s="10"/>
     </row>
-    <row r="18">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
         <v>22</v>
       </c>
@@ -1285,7 +1307,7 @@
       <c r="G18" s="9"/>
       <c r="H18" s="10"/>
     </row>
-    <row r="19">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
         <v>24</v>
       </c>
@@ -1299,7 +1321,7 @@
       <c r="G19" s="9"/>
       <c r="H19" s="10"/>
     </row>
-    <row r="20">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
         <v>26</v>
       </c>
@@ -1313,7 +1335,7 @@
       <c r="G20" s="22"/>
       <c r="H20" s="23"/>
     </row>
-    <row r="21">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
         <v>28</v>
       </c>
@@ -1327,7 +1349,7 @@
       <c r="G21" s="9"/>
       <c r="H21" s="10"/>
     </row>
-    <row r="22">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
         <v>30</v>
       </c>
@@ -1341,7 +1363,7 @@
       <c r="G22" s="9"/>
       <c r="H22" s="10"/>
     </row>
-    <row r="23">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
         <v>32</v>
       </c>
@@ -1355,7 +1377,7 @@
       <c r="G23" s="9"/>
       <c r="H23" s="10"/>
     </row>
-    <row r="24">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
         <v>34</v>
       </c>
@@ -1369,7 +1391,7 @@
       <c r="G24" s="9"/>
       <c r="H24" s="10"/>
     </row>
-    <row r="25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
         <v>36</v>
       </c>
@@ -1383,7 +1405,7 @@
       <c r="G25" s="9"/>
       <c r="H25" s="10"/>
     </row>
-    <row r="26">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
         <v>38</v>
       </c>
@@ -1397,7 +1419,7 @@
       <c r="G26" s="9"/>
       <c r="H26" s="10"/>
     </row>
-    <row r="27">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="24"/>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
@@ -1407,7 +1429,7 @@
       <c r="G27" s="9"/>
       <c r="H27" s="10"/>
     </row>
-    <row r="28">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>40</v>
       </c>
@@ -1419,7 +1441,7 @@
       <c r="G28" s="9"/>
       <c r="H28" s="10"/>
     </row>
-    <row r="29">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="25" t="s">
         <v>41</v>
       </c>
@@ -1443,7 +1465,7 @@
       </c>
       <c r="H29" s="10"/>
     </row>
-    <row r="30">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="30" t="s">
         <v>48</v>
       </c>
@@ -1467,7 +1489,7 @@
       </c>
       <c r="H30" s="10"/>
     </row>
-    <row r="31">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="30" t="s">
         <v>54</v>
       </c>
@@ -1491,7 +1513,7 @@
       </c>
       <c r="H31" s="10"/>
     </row>
-    <row r="32">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="30" t="s">
         <v>59</v>
       </c>
@@ -1515,7 +1537,7 @@
       </c>
       <c r="H32" s="10"/>
     </row>
-    <row r="33">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="30" t="s">
         <v>64</v>
       </c>
@@ -1539,7 +1561,7 @@
       </c>
       <c r="H33" s="10"/>
     </row>
-    <row r="34">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="30" t="s">
         <v>69</v>
       </c>
@@ -1563,7 +1585,7 @@
       </c>
       <c r="H34" s="10"/>
     </row>
-    <row r="35">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="30" t="s">
         <v>74</v>
       </c>
@@ -1587,7 +1609,7 @@
       </c>
       <c r="H35" s="10"/>
     </row>
-    <row r="36">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="30" t="s">
         <v>79</v>
       </c>
@@ -1611,7 +1633,7 @@
       </c>
       <c r="H36" s="10"/>
     </row>
-    <row r="37">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="30" t="s">
         <v>84</v>
       </c>
@@ -1635,7 +1657,7 @@
       </c>
       <c r="H37" s="10"/>
     </row>
-    <row r="38">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="30" t="s">
         <v>89</v>
       </c>
@@ -1659,7 +1681,7 @@
       </c>
       <c r="H38" s="10"/>
     </row>
-    <row r="39">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="30" t="s">
         <v>94</v>
       </c>
@@ -1683,7 +1705,7 @@
       </c>
       <c r="H39" s="10"/>
     </row>
-    <row r="40">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="30" t="s">
         <v>99</v>
       </c>
@@ -1707,7 +1729,7 @@
       </c>
       <c r="H40" s="10"/>
     </row>
-    <row r="41">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="30" t="s">
         <v>104</v>
       </c>
@@ -1731,7 +1753,7 @@
       </c>
       <c r="H41" s="10"/>
     </row>
-    <row r="42">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="30" t="s">
         <v>109</v>
       </c>
@@ -1755,7 +1777,7 @@
       </c>
       <c r="H42" s="10"/>
     </row>
-    <row r="43">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="30" t="s">
         <v>114</v>
       </c>
@@ -1779,7 +1801,7 @@
       </c>
       <c r="H43" s="10"/>
     </row>
-    <row r="44">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="30" t="s">
         <v>119</v>
       </c>
@@ -1803,7 +1825,7 @@
       </c>
       <c r="H44" s="10"/>
     </row>
-    <row r="45">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="32"/>
       <c r="B45" s="9"/>
       <c r="C45" s="9"/>
@@ -1813,7 +1835,7 @@
       <c r="G45" s="9"/>
       <c r="H45" s="10"/>
     </row>
-    <row r="46">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="33" t="s">
         <v>124</v>
       </c>
@@ -1825,7 +1847,7 @@
       <c r="G46" s="9"/>
       <c r="H46" s="10"/>
     </row>
-    <row r="47">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="32" t="s">
         <v>41</v>
       </c>
@@ -1839,7 +1861,7 @@
       <c r="G47" s="9"/>
       <c r="H47" s="10"/>
     </row>
-    <row r="48">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="32" t="s">
         <v>42</v>
       </c>
@@ -1853,7 +1875,7 @@
       <c r="G48" s="9"/>
       <c r="H48" s="10"/>
     </row>
-    <row r="49">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="32" t="s">
         <v>127</v>
       </c>
@@ -1867,7 +1889,7 @@
       <c r="G49" s="9"/>
       <c r="H49" s="10"/>
     </row>
-    <row r="50">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="32" t="s">
         <v>129</v>
       </c>
@@ -1881,7 +1903,7 @@
       <c r="G50" s="34"/>
       <c r="H50" s="35"/>
     </row>
-    <row r="51">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="32" t="s">
         <v>131</v>
       </c>
@@ -1895,7 +1917,7 @@
       <c r="G51" s="22"/>
       <c r="H51" s="23"/>
     </row>
-    <row r="52">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="32" t="s">
         <v>133</v>
       </c>
@@ -1909,7 +1931,7 @@
       <c r="G52" s="9"/>
       <c r="H52" s="10"/>
     </row>
-    <row r="53">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="32" t="s">
         <v>135</v>
       </c>
@@ -1923,7 +1945,7 @@
       <c r="G53" s="9"/>
       <c r="H53" s="10"/>
     </row>
-    <row r="54">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="32" t="s">
         <v>137</v>
       </c>
@@ -1937,7 +1959,7 @@
       <c r="G54" s="9"/>
       <c r="H54" s="10"/>
     </row>
-    <row r="55">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="32" t="s">
         <v>139</v>
       </c>
@@ -1951,7 +1973,7 @@
       <c r="G55" s="9"/>
       <c r="H55" s="10"/>
     </row>
-    <row r="56">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="36"/>
       <c r="B56" s="9"/>
       <c r="C56" s="9"/>
@@ -1961,7 +1983,7 @@
       <c r="G56" s="9"/>
       <c r="H56" s="10"/>
     </row>
-    <row r="57">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="33" t="s">
         <v>140</v>
       </c>
@@ -1973,7 +1995,7 @@
       <c r="G57" s="9"/>
       <c r="H57" s="10"/>
     </row>
-    <row r="58">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="37" t="s">
         <v>141</v>
       </c>
@@ -1985,39 +2007,87 @@
       <c r="G58" s="5"/>
       <c r="H58" s="6"/>
     </row>
-    <row r="59">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="7"/>
+      <c r="B59"/>
+      <c r="C59"/>
+      <c r="D59"/>
+      <c r="E59"/>
+      <c r="F59"/>
+      <c r="G59"/>
       <c r="H59" s="2"/>
     </row>
-    <row r="60">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="7"/>
+      <c r="B60"/>
+      <c r="C60"/>
+      <c r="D60"/>
+      <c r="E60"/>
+      <c r="F60"/>
+      <c r="G60"/>
       <c r="H60" s="2"/>
     </row>
-    <row r="61">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="7"/>
+      <c r="B61"/>
+      <c r="C61"/>
+      <c r="D61"/>
+      <c r="E61"/>
+      <c r="F61"/>
+      <c r="G61"/>
       <c r="H61" s="2"/>
     </row>
-    <row r="62">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="7"/>
+      <c r="B62"/>
+      <c r="C62"/>
+      <c r="D62"/>
+      <c r="E62"/>
+      <c r="F62"/>
+      <c r="G62"/>
       <c r="H62" s="2"/>
     </row>
-    <row r="63">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
+      <c r="B63"/>
+      <c r="C63"/>
+      <c r="D63"/>
+      <c r="E63"/>
+      <c r="F63"/>
+      <c r="G63"/>
       <c r="H63" s="2"/>
     </row>
-    <row r="64">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
+      <c r="B64"/>
+      <c r="C64"/>
+      <c r="D64"/>
+      <c r="E64"/>
+      <c r="F64"/>
+      <c r="G64"/>
       <c r="H64" s="2"/>
     </row>
-    <row r="65">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="7"/>
+      <c r="B65"/>
+      <c r="C65"/>
+      <c r="D65"/>
+      <c r="E65"/>
+      <c r="F65"/>
+      <c r="G65"/>
       <c r="H65" s="2"/>
     </row>
-    <row r="66">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="7"/>
+      <c r="B66"/>
+      <c r="C66"/>
+      <c r="D66"/>
+      <c r="E66"/>
+      <c r="F66"/>
+      <c r="G66"/>
       <c r="H66" s="2"/>
     </row>
-    <row r="67">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="38"/>
       <c r="B67" s="22"/>
       <c r="C67" s="22"/>
@@ -2027,7 +2097,7 @@
       <c r="G67" s="22"/>
       <c r="H67" s="23"/>
     </row>
-    <row r="68">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="33" t="s">
         <v>142</v>
       </c>
@@ -2039,7 +2109,7 @@
       <c r="G68" s="9"/>
       <c r="H68" s="10"/>
     </row>
-    <row r="69">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="39" t="s">
         <v>143</v>
       </c>
@@ -2051,39 +2121,87 @@
       <c r="G69" s="5"/>
       <c r="H69" s="6"/>
     </row>
-    <row r="70">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="7"/>
+      <c r="B70"/>
+      <c r="C70"/>
+      <c r="D70"/>
+      <c r="E70"/>
+      <c r="F70"/>
+      <c r="G70"/>
       <c r="H70" s="2"/>
     </row>
-    <row r="71">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="7"/>
+      <c r="B71"/>
+      <c r="C71"/>
+      <c r="D71"/>
+      <c r="E71"/>
+      <c r="F71"/>
+      <c r="G71"/>
       <c r="H71" s="2"/>
     </row>
-    <row r="72">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="7"/>
+      <c r="B72"/>
+      <c r="C72"/>
+      <c r="D72"/>
+      <c r="E72"/>
+      <c r="F72"/>
+      <c r="G72"/>
       <c r="H72" s="2"/>
     </row>
-    <row r="73">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="7"/>
+      <c r="B73"/>
+      <c r="C73"/>
+      <c r="D73"/>
+      <c r="E73"/>
+      <c r="F73"/>
+      <c r="G73"/>
       <c r="H73" s="2"/>
     </row>
-    <row r="74">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="7"/>
+      <c r="B74"/>
+      <c r="C74"/>
+      <c r="D74"/>
+      <c r="E74"/>
+      <c r="F74"/>
+      <c r="G74"/>
       <c r="H74" s="2"/>
     </row>
-    <row r="75">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="7"/>
+      <c r="B75"/>
+      <c r="C75"/>
+      <c r="D75"/>
+      <c r="E75"/>
+      <c r="F75"/>
+      <c r="G75"/>
       <c r="H75" s="2"/>
     </row>
-    <row r="76">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="7"/>
+      <c r="B76"/>
+      <c r="C76"/>
+      <c r="D76"/>
+      <c r="E76"/>
+      <c r="F76"/>
+      <c r="G76"/>
       <c r="H76" s="2"/>
     </row>
-    <row r="77">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="7"/>
+      <c r="B77"/>
+      <c r="C77"/>
+      <c r="D77"/>
+      <c r="E77"/>
+      <c r="F77"/>
+      <c r="G77"/>
       <c r="H77" s="2"/>
     </row>
-    <row r="78">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="38"/>
       <c r="B78" s="22"/>
       <c r="C78" s="22"/>
@@ -2093,7 +2211,7 @@
       <c r="G78" s="22"/>
       <c r="H78" s="23"/>
     </row>
-    <row r="79">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="40" t="s">
         <v>144</v>
       </c>
@@ -2105,7 +2223,7 @@
       <c r="G79" s="9"/>
       <c r="H79" s="10"/>
     </row>
-    <row r="80">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="41" t="s">
         <v>145</v>
       </c>
@@ -2117,39 +2235,87 @@
       <c r="G80" s="5"/>
       <c r="H80" s="6"/>
     </row>
-    <row r="81">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="7"/>
+      <c r="B81"/>
+      <c r="C81"/>
+      <c r="D81"/>
+      <c r="E81"/>
+      <c r="F81"/>
+      <c r="G81"/>
       <c r="H81" s="2"/>
     </row>
-    <row r="82">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="7"/>
+      <c r="B82"/>
+      <c r="C82"/>
+      <c r="D82"/>
+      <c r="E82"/>
+      <c r="F82"/>
+      <c r="G82"/>
       <c r="H82" s="2"/>
     </row>
-    <row r="83">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="7"/>
+      <c r="B83"/>
+      <c r="C83"/>
+      <c r="D83"/>
+      <c r="E83"/>
+      <c r="F83"/>
+      <c r="G83"/>
       <c r="H83" s="2"/>
     </row>
-    <row r="84">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" s="7"/>
+      <c r="B84"/>
+      <c r="C84"/>
+      <c r="D84"/>
+      <c r="E84"/>
+      <c r="F84"/>
+      <c r="G84"/>
       <c r="H84" s="2"/>
     </row>
-    <row r="85">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" s="7"/>
+      <c r="B85"/>
+      <c r="C85"/>
+      <c r="D85"/>
+      <c r="E85"/>
+      <c r="F85"/>
+      <c r="G85"/>
       <c r="H85" s="2"/>
     </row>
-    <row r="86">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" s="7"/>
+      <c r="B86"/>
+      <c r="C86"/>
+      <c r="D86"/>
+      <c r="E86"/>
+      <c r="F86"/>
+      <c r="G86"/>
       <c r="H86" s="2"/>
     </row>
-    <row r="87">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" s="7"/>
+      <c r="B87"/>
+      <c r="C87"/>
+      <c r="D87"/>
+      <c r="E87"/>
+      <c r="F87"/>
+      <c r="G87"/>
       <c r="H87" s="2"/>
     </row>
-    <row r="88">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="7"/>
+      <c r="B88"/>
+      <c r="C88"/>
+      <c r="D88"/>
+      <c r="E88"/>
+      <c r="F88"/>
+      <c r="G88"/>
       <c r="H88" s="2"/>
     </row>
-    <row r="89">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="38"/>
       <c r="B89" s="22"/>
       <c r="C89" s="22"/>
@@ -2159,7 +2325,7 @@
       <c r="G89" s="22"/>
       <c r="H89" s="23"/>
     </row>
-    <row r="90">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" s="40" t="s">
         <v>146</v>
       </c>
@@ -2171,7 +2337,7 @@
       <c r="G90" s="9"/>
       <c r="H90" s="10"/>
     </row>
-    <row r="91">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" s="41" t="s">
         <v>147</v>
       </c>
@@ -2183,39 +2349,87 @@
       <c r="G91" s="5"/>
       <c r="H91" s="6"/>
     </row>
-    <row r="92">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" s="7"/>
+      <c r="B92"/>
+      <c r="C92"/>
+      <c r="D92"/>
+      <c r="E92"/>
+      <c r="F92"/>
+      <c r="G92"/>
       <c r="H92" s="2"/>
     </row>
-    <row r="93">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" s="7"/>
+      <c r="B93"/>
+      <c r="C93"/>
+      <c r="D93"/>
+      <c r="E93"/>
+      <c r="F93"/>
+      <c r="G93"/>
       <c r="H93" s="2"/>
     </row>
-    <row r="94">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" s="7"/>
+      <c r="B94"/>
+      <c r="C94"/>
+      <c r="D94"/>
+      <c r="E94"/>
+      <c r="F94"/>
+      <c r="G94"/>
       <c r="H94" s="2"/>
     </row>
-    <row r="95">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" s="7"/>
+      <c r="B95"/>
+      <c r="C95"/>
+      <c r="D95"/>
+      <c r="E95"/>
+      <c r="F95"/>
+      <c r="G95"/>
       <c r="H95" s="2"/>
     </row>
-    <row r="96">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" s="7"/>
+      <c r="B96"/>
+      <c r="C96"/>
+      <c r="D96"/>
+      <c r="E96"/>
+      <c r="F96"/>
+      <c r="G96"/>
       <c r="H96" s="2"/>
     </row>
-    <row r="97">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" s="7"/>
+      <c r="B97"/>
+      <c r="C97"/>
+      <c r="D97"/>
+      <c r="E97"/>
+      <c r="F97"/>
+      <c r="G97"/>
       <c r="H97" s="2"/>
     </row>
-    <row r="98">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="7"/>
+      <c r="B98"/>
+      <c r="C98"/>
+      <c r="D98"/>
+      <c r="E98"/>
+      <c r="F98"/>
+      <c r="G98"/>
       <c r="H98" s="2"/>
     </row>
-    <row r="99">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" s="7"/>
+      <c r="B99"/>
+      <c r="C99"/>
+      <c r="D99"/>
+      <c r="E99"/>
+      <c r="F99"/>
+      <c r="G99"/>
       <c r="H99" s="2"/>
     </row>
-    <row r="100">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" s="38"/>
       <c r="B100" s="22"/>
       <c r="C100" s="22"/>
@@ -2225,7 +2439,7 @@
       <c r="G100" s="22"/>
       <c r="H100" s="23"/>
     </row>
-    <row r="101">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" s="40" t="s">
         <v>148</v>
       </c>
@@ -2237,7 +2451,7 @@
       <c r="G101" s="9"/>
       <c r="H101" s="10"/>
     </row>
-    <row r="102">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" s="41" t="s">
         <v>149</v>
       </c>
@@ -2249,35 +2463,77 @@
       <c r="G102" s="5"/>
       <c r="H102" s="6"/>
     </row>
-    <row r="103">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" s="7"/>
+      <c r="B103"/>
+      <c r="C103"/>
+      <c r="D103"/>
+      <c r="E103"/>
+      <c r="F103"/>
+      <c r="G103"/>
       <c r="H103" s="2"/>
     </row>
-    <row r="104">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" s="7"/>
+      <c r="B104"/>
+      <c r="C104"/>
+      <c r="D104"/>
+      <c r="E104"/>
+      <c r="F104"/>
+      <c r="G104"/>
       <c r="H104" s="2"/>
     </row>
-    <row r="105">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" s="7"/>
+      <c r="B105"/>
+      <c r="C105"/>
+      <c r="D105"/>
+      <c r="E105"/>
+      <c r="F105"/>
+      <c r="G105"/>
       <c r="H105" s="2"/>
     </row>
-    <row r="106">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" s="7"/>
+      <c r="B106"/>
+      <c r="C106"/>
+      <c r="D106"/>
+      <c r="E106"/>
+      <c r="F106"/>
+      <c r="G106"/>
       <c r="H106" s="2"/>
     </row>
-    <row r="107">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" s="7"/>
+      <c r="B107"/>
+      <c r="C107"/>
+      <c r="D107"/>
+      <c r="E107"/>
+      <c r="F107"/>
+      <c r="G107"/>
       <c r="H107" s="2"/>
     </row>
-    <row r="108">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" s="7"/>
+      <c r="B108"/>
+      <c r="C108"/>
+      <c r="D108"/>
+      <c r="E108"/>
+      <c r="F108"/>
+      <c r="G108"/>
       <c r="H108" s="2"/>
     </row>
-    <row r="109">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" s="7"/>
+      <c r="B109"/>
+      <c r="C109"/>
+      <c r="D109"/>
+      <c r="E109"/>
+      <c r="F109"/>
+      <c r="G109"/>
       <c r="H109" s="2"/>
     </row>
-    <row r="110">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" s="38"/>
       <c r="B110" s="22"/>
       <c r="C110" s="22"/>
@@ -2287,7 +2543,7 @@
       <c r="G110" s="22"/>
       <c r="H110" s="23"/>
     </row>
-    <row r="111">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" s="42"/>
       <c r="B111" s="43"/>
       <c r="C111" s="43"/>
@@ -2297,7 +2553,7 @@
       <c r="G111" s="43"/>
       <c r="H111" s="44"/>
     </row>
-    <row r="112">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" s="45" t="s">
         <v>150</v>
       </c>
@@ -2309,7 +2565,7 @@
       <c r="G112" s="43"/>
       <c r="H112" s="44"/>
     </row>
-    <row r="113">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" s="45"/>
       <c r="B113" s="43"/>
       <c r="C113" s="43"/>
@@ -2319,10 +2575,11 @@
       <c r="G113" s="43"/>
       <c r="H113" s="44"/>
     </row>
-    <row r="114">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" s="46" t="s">
         <v>151</v>
       </c>
+      <c r="B114"/>
       <c r="C114" s="43"/>
       <c r="D114" s="43"/>
       <c r="E114" s="43"/>
@@ -2330,7 +2587,7 @@
       <c r="G114" s="43"/>
       <c r="H114" s="44"/>
     </row>
-    <row r="115">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" s="47" t="s">
         <v>152</v>
       </c>
@@ -2342,7 +2599,7 @@
       <c r="G115" s="43"/>
       <c r="H115" s="44"/>
     </row>
-    <row r="116">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" s="48"/>
       <c r="B116" s="48"/>
       <c r="C116" s="43"/>
@@ -2352,7 +2609,7 @@
       <c r="G116" s="43"/>
       <c r="H116" s="44"/>
     </row>
-    <row r="117">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" s="49"/>
       <c r="B117" s="49"/>
       <c r="C117" s="50"/>
@@ -2364,6 +2621,55 @@
     </row>
   </sheetData>
   <mergeCells count="92">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:H8"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="G33:H33"/>
+    <mergeCell ref="G34:H34"/>
     <mergeCell ref="G35:H35"/>
     <mergeCell ref="G36:H36"/>
     <mergeCell ref="G37:H37"/>
@@ -2378,28 +2684,25 @@
     <mergeCell ref="A46:H46"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="D47:H47"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="A52:C52"/>
-    <mergeCell ref="A53:C53"/>
-    <mergeCell ref="A54:C54"/>
-    <mergeCell ref="A55:C55"/>
     <mergeCell ref="A48:C48"/>
     <mergeCell ref="D48:H48"/>
     <mergeCell ref="A49:C49"/>
     <mergeCell ref="D49:H49"/>
     <mergeCell ref="A50:C50"/>
     <mergeCell ref="D50:F50"/>
+    <mergeCell ref="A51:C51"/>
     <mergeCell ref="D51:H51"/>
+    <mergeCell ref="A52:C52"/>
     <mergeCell ref="D52:H52"/>
+    <mergeCell ref="A53:C53"/>
     <mergeCell ref="D53:H53"/>
+    <mergeCell ref="A54:C54"/>
     <mergeCell ref="D54:H54"/>
+    <mergeCell ref="A55:C55"/>
     <mergeCell ref="D55:H55"/>
     <mergeCell ref="A56:H56"/>
     <mergeCell ref="A57:H57"/>
     <mergeCell ref="A58:H67"/>
-    <mergeCell ref="A102:H110"/>
-    <mergeCell ref="A115:B115"/>
-    <mergeCell ref="A114:B114"/>
     <mergeCell ref="A68:H68"/>
     <mergeCell ref="A69:H78"/>
     <mergeCell ref="A79:H79"/>
@@ -2407,56 +2710,9 @@
     <mergeCell ref="A90:H90"/>
     <mergeCell ref="A91:H100"/>
     <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:H8"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A28:H28"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="G33:H33"/>
-    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="A102:H110"/>
+    <mergeCell ref="A114:B114"/>
+    <mergeCell ref="A115:B115"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>